<commit_message>
Added training material links
</commit_message>
<xml_diff>
--- a/GenAI Learning Roadmap.xlsx
+++ b/GenAI Learning Roadmap.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\267564\OneDrive - NTT Data Group\ValueX\GitRepos\Documents\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CED7E9C3-A21C-439C-8668-9356F0657424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F281883C-1BD1-4945-9432-90F167A1DBCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{1684B1F0-1F6A-4729-96C5-DDAA8F3EA7A9}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{1684B1F0-1F6A-4729-96C5-DDAA8F3EA7A9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="71">
   <si>
     <t>Topics</t>
   </si>
@@ -234,13 +234,31 @@
   </si>
   <si>
     <t>Complete the training to understand fundamental GenAI implementatinos using bedrock</t>
+  </si>
+  <si>
+    <t>https://cloud.google.com/use-cases/retrieval-augmented-generation</t>
+  </si>
+  <si>
+    <t>What are Embeddings and how do it work?</t>
+  </si>
+  <si>
+    <t>https://medium.com/@eugenesh4work/what-are-embeddings-and-how-do-it-work-b35af573b59e</t>
+  </si>
+  <si>
+    <t>https://learn.microsoft.com/en-us/data-engineering/playbook/solutions/vector-database/</t>
+  </si>
+  <si>
+    <t>Lanchain intro and basics</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=J_0qvRt4LNk</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -269,12 +287,6 @@
       <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -320,7 +332,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -330,9 +342,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -818,7 +827,7 @@
       </c>
       <c r="H6" s="4"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -826,27 +835,33 @@
         <v>23</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="D7" s="2" t="s">
+        <v>65</v>
+      </c>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="C8" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>67</v>
+      </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -854,21 +869,27 @@
         <v>25</v>
       </c>
       <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="D9" s="2" t="s">
+        <v>68</v>
+      </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
+      <c r="C10" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>70</v>
+      </c>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
@@ -907,7 +928,7 @@
       <c r="F12" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="1" t="s">
         <v>32</v>
       </c>
       <c r="H12" s="4"/>
@@ -925,13 +946,13 @@
       <c r="D13" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="5" t="s">
         <v>42</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="1" t="s">
         <v>44</v>
       </c>
       <c r="H13" s="4"/>
@@ -1013,7 +1034,7 @@
       <c r="D18" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="5" t="s">
         <v>42</v>
       </c>
       <c r="F18" s="1" t="s">
@@ -1072,16 +1093,20 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D4" r:id="rId1" xr:uid="{DE7C3A35-CA96-4871-8987-2FB228113558}"/>
-    <hyperlink ref="D6" r:id="rId2" xr:uid="{2E67737B-B2ED-4166-96F8-603FED4E569E}"/>
-    <hyperlink ref="D13" r:id="rId3" xr:uid="{FEBBBC1D-1339-49A3-B234-A52314FCF19A}"/>
-    <hyperlink ref="E13" r:id="rId4" display="https://www.youtube.com/@samwitteveenai" xr:uid="{BD1030F5-4D0C-444F-9DFA-7514118FD6B2}"/>
-    <hyperlink ref="D12" r:id="rId5" xr:uid="{7ABA2D64-DEC2-407E-BDC1-3E6D1664D307}"/>
-    <hyperlink ref="D14" r:id="rId6" xr:uid="{9975E14A-E0E0-45FA-894A-4ABE81A32C12}"/>
-    <hyperlink ref="E18" r:id="rId7" display="https://www.youtube.com/@samwitteveenai" xr:uid="{A2C02E57-EC9D-4192-85BC-6F788953B21B}"/>
-    <hyperlink ref="D20" r:id="rId8" xr:uid="{3D44D625-C2FB-4D57-9548-31F87BD2405A}"/>
-    <hyperlink ref="D18" r:id="rId9" xr:uid="{3DA61AAD-4B06-4A57-BAF7-9B6B4D5F03DD}"/>
-    <hyperlink ref="D3" r:id="rId10" location="content" xr:uid="{E51736A3-B398-4941-B7A8-A3D757531B4F}"/>
+    <hyperlink ref="D4" r:id="rId1" xr:uid="{376998E4-6FED-40F1-B6B3-361DF31D9A54}"/>
+    <hyperlink ref="D6" r:id="rId2" xr:uid="{251DCB06-1FBB-46E7-81BD-F14E2657218C}"/>
+    <hyperlink ref="D13" r:id="rId3" xr:uid="{635097EE-C272-4778-A3DC-C646A9C129D9}"/>
+    <hyperlink ref="E13" r:id="rId4" display="https://www.youtube.com/@samwitteveenai" xr:uid="{C23EC549-9885-4B4B-9050-E52F6593E736}"/>
+    <hyperlink ref="D12" r:id="rId5" xr:uid="{44F28B66-F120-4804-8609-160870514B23}"/>
+    <hyperlink ref="D14" r:id="rId6" xr:uid="{8A30DA20-1194-4C43-BEB6-139EA8529854}"/>
+    <hyperlink ref="E18" r:id="rId7" display="https://www.youtube.com/@samwitteveenai" xr:uid="{5BF7098E-FAFF-4B9F-A50B-75776947291D}"/>
+    <hyperlink ref="D20" r:id="rId8" xr:uid="{EB0A5EFC-D098-4FDB-B087-FC01DAE2C46F}"/>
+    <hyperlink ref="D18" r:id="rId9" xr:uid="{9960C19D-C231-4D34-8B44-D7146DECE135}"/>
+    <hyperlink ref="D3" r:id="rId10" location="content" xr:uid="{6D5B8E86-4787-4C09-9AA0-1DEE45EA8B23}"/>
+    <hyperlink ref="D9" r:id="rId11" xr:uid="{8E07A8FE-C1FA-49E0-90C8-798BCC90D506}"/>
+    <hyperlink ref="D8" r:id="rId12" xr:uid="{19322042-DAF9-4C31-BD0E-7EBC7D498900}"/>
+    <hyperlink ref="D7" r:id="rId13" xr:uid="{9A7B78B0-998A-4606-AA75-473867956BB5}"/>
+    <hyperlink ref="D10" r:id="rId14" xr:uid="{CF897636-27B6-49B7-9DE5-F7DAC4C565D7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>